<commit_message>
Mise à jour reconciliation et mapping Wave
</commit_message>
<xml_diff>
--- a/data/mappings/mapping_agences_cofina_wave.xlsx
+++ b/data/mappings/mapping_agences_cofina_wave.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\haby.sow\Downloads\reconciliation-main\reconciliation-main\data\mappings\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\haby.sow\Downloads\reconciliation-git\data\mappings\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2FA2F44-B470-41F8-82D5-399274F26560}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7996C209-C9FF-425A-B361-B882090ED050}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,14 +16,14 @@
     <sheet name="Sheet" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet!$A$1:$C$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet!$A$1:$C$39</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="58">
   <si>
     <t>CODE_AGENCE</t>
   </si>
@@ -194,6 +194,9 @@
   </si>
   <si>
     <t>AGENCE KEUR MASSAR</t>
+  </si>
+  <si>
+    <t>Master Cofina Express Pikine</t>
   </si>
 </sst>
 </file>
@@ -546,7 +549,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C39"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="27.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -564,7 +568,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2"/>
       <c r="B2">
         <v>535</v>
@@ -573,7 +577,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>48</v>
       </c>
@@ -584,7 +588,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
@@ -595,7 +599,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>45</v>
       </c>
@@ -606,7 +610,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>36</v>
       </c>
@@ -617,7 +621,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>30</v>
       </c>
@@ -628,7 +632,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
@@ -639,7 +643,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>39</v>
       </c>
@@ -650,7 +654,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
@@ -661,183 +665,183 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B11">
-        <v>504</v>
+        <v>510</v>
       </c>
       <c r="C11" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A12" s="2" t="s">
-        <v>42</v>
-      </c>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="2"/>
       <c r="B12">
-        <v>510</v>
+        <v>540</v>
       </c>
       <c r="C12" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" s="2"/>
       <c r="B13">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="C13" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" s="2"/>
       <c r="B14">
-        <v>541</v>
+        <v>533</v>
       </c>
       <c r="C14" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A15" s="2"/>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="2" t="s">
+        <v>54</v>
+      </c>
       <c r="B15">
-        <v>533</v>
+        <v>524</v>
       </c>
       <c r="C15" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16">
+        <v>512</v>
+      </c>
+      <c r="C16" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B17">
+        <v>503</v>
+      </c>
+      <c r="C17" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="2"/>
+      <c r="B18">
+        <v>534</v>
+      </c>
+      <c r="C18" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B16">
+      <c r="B19">
         <v>524</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C19" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A17" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B17">
-        <v>512</v>
-      </c>
-      <c r="C17" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A18" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B18">
-        <v>503</v>
-      </c>
-      <c r="C18" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A19" s="2"/>
-      <c r="B19">
-        <v>534</v>
-      </c>
-      <c r="C19" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
-        <v>54</v>
+        <v>28</v>
       </c>
       <c r="B20">
-        <v>524</v>
+        <v>505</v>
       </c>
       <c r="C20" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="B21">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="C21" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B22">
-        <v>508</v>
+        <v>502</v>
       </c>
       <c r="C22" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="B23">
-        <v>502</v>
+        <v>518</v>
       </c>
       <c r="C23" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
-        <v>50</v>
+        <v>19</v>
       </c>
       <c r="B24">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="C24" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
-        <v>19</v>
+        <v>49</v>
       </c>
       <c r="B25">
-        <v>516</v>
+        <v>511</v>
       </c>
       <c r="C25" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="B26">
-        <v>511</v>
+        <v>501</v>
       </c>
       <c r="C26" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B27">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="C27" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.35">
@@ -851,7 +855,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>44</v>
       </c>
@@ -862,7 +866,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>41</v>
       </c>
@@ -873,7 +877,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>47</v>
       </c>
@@ -884,7 +888,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>46</v>
       </c>
@@ -895,7 +899,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>28</v>
       </c>
@@ -906,7 +910,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>30</v>
       </c>
@@ -917,7 +921,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>52</v>
       </c>
@@ -928,7 +932,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="B36">
         <v>539</v>
       </c>
@@ -936,7 +940,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>39</v>
       </c>
@@ -947,7 +951,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>53</v>
       </c>
@@ -958,7 +962,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>55</v>
       </c>
@@ -969,8 +973,25 @@
         <v>56</v>
       </c>
     </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>57</v>
+      </c>
+      <c r="B40">
+        <v>504</v>
+      </c>
+      <c r="C40" t="s">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:C39" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="504"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Mise a jour reconciliation PI SPI et nettoyage Git
</commit_message>
<xml_diff>
--- a/data/mappings/mapping_agences_cofina_wave.xlsx
+++ b/data/mappings/mapping_agences_cofina_wave.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\haby.sow\Downloads\reconciliation-git\data\mappings\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7996C209-C9FF-425A-B361-B882090ED050}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F51D1F03-8DF5-4206-8E10-25FE015645F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,14 +16,14 @@
     <sheet name="Sheet" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet!$A$1:$C$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet!$A$1:$C$38</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="57">
   <si>
     <t>CODE_AGENCE</t>
   </si>
@@ -145,9 +145,6 @@
     <t>Master Cofina Express LINGUER'LA</t>
   </si>
   <si>
-    <t>*Cofina Express Pikine*</t>
-  </si>
-  <si>
     <t xml:space="preserve">Cofina Thiès </t>
   </si>
   <si>
@@ -196,7 +193,7 @@
     <t>AGENCE KEUR MASSAR</t>
   </si>
   <si>
-    <t>Master Cofina Express Pikine</t>
+    <t>Cofina Pikine 2</t>
   </si>
 </sst>
 </file>
@@ -243,10 +240,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -550,7 +548,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:D49"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="27.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -579,7 +577,7 @@
     </row>
     <row r="3" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B3">
         <v>519</v>
@@ -601,7 +599,7 @@
     </row>
     <row r="5" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B5">
         <v>517</v>
@@ -667,7 +665,7 @@
     </row>
     <row r="11" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B11">
         <v>510</v>
@@ -705,7 +703,7 @@
     </row>
     <row r="15" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B15">
         <v>524</v>
@@ -747,7 +745,7 @@
     </row>
     <row r="19" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B19">
         <v>524</v>
@@ -769,7 +767,7 @@
     </row>
     <row r="21" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B21">
         <v>508</v>
@@ -791,7 +789,7 @@
     </row>
     <row r="23" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B23">
         <v>518</v>
@@ -813,7 +811,7 @@
     </row>
     <row r="25" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B25">
         <v>511</v>
@@ -824,7 +822,7 @@
     </row>
     <row r="26" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B26">
         <v>501</v>
@@ -835,7 +833,7 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="B27">
         <v>504</v>
@@ -844,148 +842,140 @@
         <v>23</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A28" s="2" t="s">
-        <v>51</v>
+    <row r="28" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>43</v>
       </c>
       <c r="B28">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="C28" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="29" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B29">
-        <v>502</v>
+        <v>508</v>
       </c>
       <c r="C29" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="30" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="B30">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="C30" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="31" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B31">
-        <v>506</v>
+        <v>503</v>
       </c>
       <c r="C31" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="32" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="B32">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="C32" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="33" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B33">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="C33" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="34" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>30</v>
+        <v>51</v>
       </c>
       <c r="B34">
-        <v>507</v>
+        <v>517</v>
       </c>
       <c r="C34" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="35" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A35" t="s">
-        <v>52</v>
-      </c>
       <c r="B35">
-        <v>517</v>
+        <v>539</v>
       </c>
       <c r="C35" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="36" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>39</v>
+      </c>
       <c r="B36">
-        <v>539</v>
+        <v>525</v>
       </c>
       <c r="C36" t="s">
-        <v>33</v>
+        <v>7</v>
       </c>
     </row>
     <row r="37" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="B37">
-        <v>525</v>
+        <v>543</v>
       </c>
       <c r="C37" t="s">
-        <v>7</v>
+        <v>34</v>
       </c>
     </row>
     <row r="38" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B38">
-        <v>543</v>
+        <v>527</v>
       </c>
       <c r="C38" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B39">
-        <v>527</v>
+        <v>504</v>
       </c>
       <c r="C39" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A40" t="s">
-        <v>57</v>
-      </c>
-      <c r="B40">
-        <v>504</v>
-      </c>
-      <c r="C40" t="s">
         <v>23</v>
       </c>
     </row>
+    <row r="49" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D49" s="3"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C39" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <autoFilter ref="A1:C38" xr:uid="{00000000-0001-0000-0000-000000000000}">
     <filterColumn colId="1">
       <filters>
         <filter val="504"/>

</xml_diff>